<commit_message>
feat(catalog): restore LSC101-108 10 oz Polar Camel Sippy Cups
- Remove the 8 SKUs from REMOVED_SKUS (operator request, 2026-07-20)
- Price list: 8 rows at $9.10 blank + $4 front + $2 back + $1 handling
- Weights (0.92 lb) and shipping dims (7 x 5 x 5 in, engrave 69.9 x 82.6 mm)
  sourced from JDS product page (case qty 24, individually packaged)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/FomaPrint-Price-List.xlsx
+++ b/public/FomaPrint-Price-List.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SKU list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU list" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O842"/>
+  <dimension ref="A1:O850"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -50910,6 +50910,494 @@
         <v/>
       </c>
     </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>LSC101</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E843" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>Black 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J843" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K843" t="n">
+        <v>4</v>
+      </c>
+      <c r="L843" t="n">
+        <v>2</v>
+      </c>
+      <c r="M843" t="n">
+        <v>1</v>
+      </c>
+      <c r="N843">
+        <f>J843+K843+M843</f>
+        <v/>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>LSC102</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E844" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>Red 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J844" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K844" t="n">
+        <v>4</v>
+      </c>
+      <c r="L844" t="n">
+        <v>2</v>
+      </c>
+      <c r="M844" t="n">
+        <v>1</v>
+      </c>
+      <c r="N844">
+        <f>J844+K844+M844</f>
+        <v/>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>LSC103</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Royal Blue</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E845" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>Royal Blue 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J845" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K845" t="n">
+        <v>4</v>
+      </c>
+      <c r="L845" t="n">
+        <v>2</v>
+      </c>
+      <c r="M845" t="n">
+        <v>1</v>
+      </c>
+      <c r="N845">
+        <f>J845+K845+M845</f>
+        <v/>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>LSC104</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E846" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>Pink 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J846" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K846" t="n">
+        <v>4</v>
+      </c>
+      <c r="L846" t="n">
+        <v>2</v>
+      </c>
+      <c r="M846" t="n">
+        <v>1</v>
+      </c>
+      <c r="N846">
+        <f>J846+K846+M846</f>
+        <v/>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>LSC105</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E847" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>Teal 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J847" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K847" t="n">
+        <v>4</v>
+      </c>
+      <c r="L847" t="n">
+        <v>2</v>
+      </c>
+      <c r="M847" t="n">
+        <v>1</v>
+      </c>
+      <c r="N847">
+        <f>J847+K847+M847</f>
+        <v/>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>LSC106</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Light Blue</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E848" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>Light Blue 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J848" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K848" t="n">
+        <v>4</v>
+      </c>
+      <c r="L848" t="n">
+        <v>2</v>
+      </c>
+      <c r="M848" t="n">
+        <v>1</v>
+      </c>
+      <c r="N848">
+        <f>J848+K848+M848</f>
+        <v/>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>LSC107</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E849" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>White 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J849" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K849" t="n">
+        <v>4</v>
+      </c>
+      <c r="L849" t="n">
+        <v>2</v>
+      </c>
+      <c r="M849" t="n">
+        <v>1</v>
+      </c>
+      <c r="N849">
+        <f>J849+K849+M849</f>
+        <v/>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>LSC108</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Olive Green</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E850" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>Olive Green 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J850" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K850" t="n">
+        <v>4</v>
+      </c>
+      <c r="L850" t="n">
+        <v>2</v>
+      </c>
+      <c r="M850" t="n">
+        <v>1</v>
+      </c>
+      <c r="N850">
+        <f>J850+K850+M850</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(catalog): restore LSC101-108 10 oz Polar Camel Sippy Cups (#46)
- Remove the 8 SKUs from REMOVED_SKUS (operator request, 2026-07-20)
- Price list: 8 rows at $9.10 blank + $4 front + $2 back + $1 handling
- Weights (0.92 lb) and shipping dims (7 x 5 x 5 in, engrave 69.9 x 82.6 mm)
  sourced from JDS product page (case qty 24, individually packaged)

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/FomaPrint-Price-List.xlsx
+++ b/public/FomaPrint-Price-List.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SKU list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SKU list" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O842"/>
+  <dimension ref="A1:O850"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -50910,6 +50910,494 @@
         <v/>
       </c>
     </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>LSC101</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E843" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>Black 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J843" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K843" t="n">
+        <v>4</v>
+      </c>
+      <c r="L843" t="n">
+        <v>2</v>
+      </c>
+      <c r="M843" t="n">
+        <v>1</v>
+      </c>
+      <c r="N843">
+        <f>J843+K843+M843</f>
+        <v/>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>LSC102</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E844" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>Red 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J844" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K844" t="n">
+        <v>4</v>
+      </c>
+      <c r="L844" t="n">
+        <v>2</v>
+      </c>
+      <c r="M844" t="n">
+        <v>1</v>
+      </c>
+      <c r="N844">
+        <f>J844+K844+M844</f>
+        <v/>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>LSC103</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Royal Blue</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E845" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>Royal Blue 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J845" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K845" t="n">
+        <v>4</v>
+      </c>
+      <c r="L845" t="n">
+        <v>2</v>
+      </c>
+      <c r="M845" t="n">
+        <v>1</v>
+      </c>
+      <c r="N845">
+        <f>J845+K845+M845</f>
+        <v/>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>LSC104</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E846" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>Pink 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J846" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K846" t="n">
+        <v>4</v>
+      </c>
+      <c r="L846" t="n">
+        <v>2</v>
+      </c>
+      <c r="M846" t="n">
+        <v>1</v>
+      </c>
+      <c r="N846">
+        <f>J846+K846+M846</f>
+        <v/>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>LSC105</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Teal</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E847" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>Teal 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J847" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K847" t="n">
+        <v>4</v>
+      </c>
+      <c r="L847" t="n">
+        <v>2</v>
+      </c>
+      <c r="M847" t="n">
+        <v>1</v>
+      </c>
+      <c r="N847">
+        <f>J847+K847+M847</f>
+        <v/>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>LSC106</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Light Blue</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E848" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>Light Blue 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J848" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K848" t="n">
+        <v>4</v>
+      </c>
+      <c r="L848" t="n">
+        <v>2</v>
+      </c>
+      <c r="M848" t="n">
+        <v>1</v>
+      </c>
+      <c r="N848">
+        <f>J848+K848+M848</f>
+        <v/>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>LSC107</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E849" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>White 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J849" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K849" t="n">
+        <v>4</v>
+      </c>
+      <c r="L849" t="n">
+        <v>2</v>
+      </c>
+      <c r="M849" t="n">
+        <v>1</v>
+      </c>
+      <c r="N849">
+        <f>J849+K849+M849</f>
+        <v/>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>JDS Industries</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>LSC108</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Olive Green</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>10 oz.</t>
+        </is>
+      </c>
+      <c r="E850" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>7 × 5 × 5</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>Drinkware</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>Sippy Cups</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>Olive Green 10 oz. Polar Camel Sippy Cup</t>
+        </is>
+      </c>
+      <c r="J850" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K850" t="n">
+        <v>4</v>
+      </c>
+      <c r="L850" t="n">
+        <v>2</v>
+      </c>
+      <c r="M850" t="n">
+        <v>1</v>
+      </c>
+      <c r="N850">
+        <f>J850+K850+M850</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>